<commit_message>
chore: update daily financial AI scenarios
</commit_message>
<xml_diff>
--- a/金融業AI場景應用.xlsx
+++ b/金融業AI場景應用.xlsx
@@ -563,8 +563,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="金融業AI場景明細" displayName="金融業AI場景明細" ref="A1:F178" headerRowCount="1" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:F178"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="金融業AI場景明細" displayName="金融業AI場景明細" ref="A1:F186" headerRowCount="1" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A1:F186"/>
   <tableColumns count="6">
     <tableColumn id="1" name="業別" dataDxfId="10"/>
     <tableColumn id="2" name="業者" dataDxfId="9"/>
@@ -913,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F178"/>
+  <dimension ref="A1:F186"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11.1640625" bestFit="1" customWidth="1" style="28" min="1" max="1"/>
@@ -6266,18 +6266,258 @@
         <v>46322</v>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>證券期貨業</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>凱基證券</t>
+        </is>
+      </c>
+      <c r="C179" s="20" t="inlineStr">
+        <is>
+          <t>凱基金</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>打造「AI 投研智慧釀酒廠」，採用 Data × Skill × Cowork 架構整合資料與專家知識，由生成式 AI 自動執行研究資料蒐集、分析比對與報告產製。</t>
+        </is>
+      </c>
+      <c r="E179" s="3" t="inlineStr">
+        <is>
+          <t>生成式AI</t>
+        </is>
+      </c>
+      <c r="F179" s="37" t="n">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="3" t="inlineStr">
+        <is>
+          <t>保險業</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>凱基人壽</t>
+        </is>
+      </c>
+      <c r="C180" s="20" t="inlineStr">
+        <is>
+          <t>凱基金</t>
+        </is>
+      </c>
+      <c r="D180" s="3" t="inlineStr">
+        <is>
+          <t>自主研發「IDEA 智慧幕僚平台」，結合生成式 AI、OCR 與大數據分析落地核保、理賠、人資與風控，提供職務說明生成、會議摘要與智慧文件判讀。</t>
+        </is>
+      </c>
+      <c r="E180" s="3" t="inlineStr">
+        <is>
+          <t>生成式AI</t>
+        </is>
+      </c>
+      <c r="F180" s="37" t="n">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="3" t="inlineStr">
+        <is>
+          <t>保險業</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>國泰人壽</t>
+        </is>
+      </c>
+      <c r="C181" s="20" t="inlineStr">
+        <is>
+          <t>國泰金</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>以「LifeLink」串聯國泰人壽 App 與新業務平台（NAP），推出「AI 全能助手」與「AI 保單辨識」（辨識率達 95%），拍照或上傳即可自動建檔並產出保單健檢。</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="inlineStr">
+        <is>
+          <t>App</t>
+        </is>
+      </c>
+      <c r="F181" s="37" t="n">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>保險業</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>國泰產險</t>
+        </is>
+      </c>
+      <c r="C182" s="20" t="inlineStr">
+        <is>
+          <t>國泰金</t>
+        </is>
+      </c>
+      <c r="D182" s="3" t="inlineStr">
+        <is>
+          <t>將 AI 深度導入理賠核心流程加速單據審核與智慧估損，使估損時間效率大幅提升 83%、每年節省逾 1,000 小時工時，保戶平均提前 7 天獲得理賠。</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>其它</t>
+        </is>
+      </c>
+      <c r="F182" s="37" t="n">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="3" t="inlineStr">
+        <is>
+          <t>銀行業</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>台新銀行</t>
+        </is>
+      </c>
+      <c r="C183" s="20" t="inlineStr">
+        <is>
+          <t>台新新光金</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="inlineStr">
+        <is>
+          <t>推出「LUNA」AI 個人信貸決策模型，採多任務深度學習（MTL）結合作業研究演算法同步優化核准率、額度與利率，帶動月撥款成長近三成並節省 90% 維運人力。</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>模型訓練</t>
+        </is>
+      </c>
+      <c r="F183" s="37" t="n">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t>銀行業</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>中國信託銀行</t>
+        </is>
+      </c>
+      <c r="C184" s="20" t="inlineStr">
+        <is>
+          <t>中信金</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="inlineStr">
+        <is>
+          <t>打造小微企業「一站式智慧融資平台（SWIP）」，結合 AI 自動化查驗、數位徵審與遠距對保重構申貸流程，使申貸審查時效大幅縮短逾 70%。</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="F184" s="37" t="n">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>銀行業</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>台北富邦銀行</t>
+        </is>
+      </c>
+      <c r="C185" s="20" t="inlineStr">
+        <is>
+          <t>富邦金</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>建置「制度化即時市場風險治理與自主評價智能風控整合平台」，結合 AI 智慧監控、自主評價模型與雲端 GPU 平行運算，使衍生性商品評價與風險計算時間縮短 90%。</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>模型訓練</t>
+        </is>
+      </c>
+      <c r="F185" s="37" t="n">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>銀行業</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>永豐銀行</t>
+        </is>
+      </c>
+      <c r="C186" s="20" t="inlineStr">
+        <is>
+          <t>永豐金</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>於信貸與信用卡徵審導入「所得代理模型」，運用 AI 與大數據分析逾 470 項帳戶金流與行為參數，協助無固定薪資證明之多元職業族群完成信用評估。</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
+        <is>
+          <t>模型訓練</t>
+        </is>
+      </c>
+      <c r="F186" s="37" t="n">
+        <v>46323</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="E2:E178" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="請選擇有效類別" error="請使用下拉選單中的類別，分類項目請參閱「分類說明」。" type="list">
+    <dataValidation sqref="E2:E186" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="請選擇有效類別" error="請使用下拉選單中的類別，分類項目請參閱「分類說明」。" type="list">
       <formula1>類別選項</formula1>
     </dataValidation>
-    <dataValidation sqref="A2:A178" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="A2:A186" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>業別選項</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B178" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B186" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>業者選項</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C178" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C186" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>所屬金控選項</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>